<commit_message>
all testcases added prperly
</commit_message>
<xml_diff>
--- a/results/TestResults.xlsx
+++ b/results/TestResults.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="28">
   <si>
     <t>Test Case</t>
   </si>
@@ -23,13 +23,49 @@
     <t>Message</t>
   </si>
   <si>
+    <t>verifyFirstHospitalOpen24x7</t>
+  </si>
+  <si>
+    <t>PASS</t>
+  </si>
+  <si>
+    <t>Test passed successfully</t>
+  </si>
+  <si>
+    <t>verifyFirstHospitalWithParking</t>
+  </si>
+  <si>
+    <t>verifyHospitalRatingAbove35</t>
+  </si>
+  <si>
+    <t>findNearestEligibleHospital</t>
+  </si>
+  <si>
+    <t>findBestRatedEligibleHospital</t>
+  </si>
+  <si>
+    <t>verifyMultipleEligibleHospitals</t>
+  </si>
+  <si>
+    <t>verifyTopCitiesSectionIsDisplayed</t>
+  </si>
+  <si>
+    <t>captureTopCities</t>
+  </si>
+  <si>
+    <t>verifyTopCitiesAreUnique</t>
+  </si>
+  <si>
+    <t>verifyNavigation</t>
+  </si>
+  <si>
     <t>filterByGenderMale</t>
   </si>
   <si>
-    <t>PASS</t>
-  </si>
-  <si>
-    <t>Test passed successfully</t>
+    <t>filterByPatientStories</t>
+  </si>
+  <si>
+    <t>filterByFeesAndExperience</t>
   </si>
   <si>
     <t>DiagnosticsCityClickTest_19</t>
@@ -39,6 +75,27 @@
   </si>
   <si>
     <t>CorporateWellnessLinkTest_21</t>
+  </si>
+  <si>
+    <t>CorporateWindowSwitchTest_22</t>
+  </si>
+  <si>
+    <t>CorporateFormInvalidInputTest_23</t>
+  </si>
+  <si>
+    <t>LabTestsAddToCartTest_24</t>
+  </si>
+  <si>
+    <t>findDoctors</t>
+  </si>
+  <si>
+    <t>verifyDropdownFilters</t>
+  </si>
+  <si>
+    <t>verifyDropdownAndRadioFilters</t>
+  </si>
+  <si>
+    <t>verifyResetFilters</t>
   </si>
 </sst>
 </file>
@@ -83,7 +140,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:C5"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -141,6 +198,226 @@
         <v>5</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C21" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>24</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C23" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s" s="0">
+        <v>26</v>
+      </c>
+      <c r="B24" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C25" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>